<commit_message>
Corrida | SFE-EIP2 | 2026-05-22 09:51:31.232411
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EIP2_out.xlsx
+++ b/indicadores/SFE-EIP2_out.xlsx
@@ -107,13 +107,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">23/04/2026</t>
+    <t xml:space="preserve">22/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1508,7 +1508,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.403490042090018</v>
+        <v>0.396520988863073</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1566,7 +1566,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.162804214065804</v>
+        <v>0.157228894608949</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1636,7 +1636,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.0504597601901364</v>
+        <v>0.253509355099073</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1666,7 +1666,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.049952433643187</v>
+        <v>0.0316479676060023</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -13547,7 +13547,7 @@
         <v>301</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.180685354825543</v>
+        <v>-0.187251838218417</v>
       </c>
     </row>
     <row r="6">
@@ -13555,7 +13555,7 @@
         <v>302</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.200575595947131</v>
+        <v>-0.198147797308738</v>
       </c>
     </row>
     <row r="7">
@@ -13563,7 +13563,7 @@
         <v>303</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.213542784742094</v>
+        <v>-0.203866170889332</v>
       </c>
     </row>
     <row r="8">
@@ -13571,7 +13571,7 @@
         <v>304</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.20659388318656</v>
+        <v>-0.192186064595916</v>
       </c>
     </row>
     <row r="9">
@@ -13579,7 +13579,7 @@
         <v>305</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.130649779245453</v>
+        <v>-0.122566490927507</v>
       </c>
     </row>
     <row r="10">
@@ -13587,7 +13587,7 @@
         <v>306</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.0174696093768747</v>
+        <v>0.00750530486887774</v>
       </c>
     </row>
     <row r="11">
@@ -13595,7 +13595,7 @@
         <v>307</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.15017109527723</v>
+        <v>0.13759568433841</v>
       </c>
     </row>
     <row r="12">
@@ -13603,7 +13603,7 @@
         <v>308</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.278730831323927</v>
+        <v>0.272651807557375</v>
       </c>
     </row>
     <row r="13">
@@ -13611,7 +13611,7 @@
         <v>309</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.40054443413837</v>
+        <v>0.390290466737657</v>
       </c>
     </row>
     <row r="14">
@@ -13619,7 +13619,7 @@
         <v>310</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.403490042090018</v>
+        <v>0.396520988863073</v>
       </c>
     </row>
     <row r="15">
@@ -13627,7 +13627,7 @@
         <v>311</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.324082310279452</v>
+        <v>0.34139738342339</v>
       </c>
     </row>
     <row r="16">
@@ -13635,7 +13635,7 @@
         <v>312</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.295837873454208</v>
+        <v>0.311862138013072</v>
       </c>
     </row>
     <row r="17">
@@ -13643,7 +13643,7 @@
         <v>313</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.278948009629394</v>
+        <v>0.283985647960897</v>
       </c>
     </row>
     <row r="18">
@@ -13651,7 +13651,7 @@
         <v>314</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.244954548249057</v>
+        <v>0.239011658315585</v>
       </c>
     </row>
     <row r="19">
@@ -13659,7 +13659,7 @@
         <v>315</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.188637832360201</v>
+        <v>0.183726426448297</v>
       </c>
     </row>
     <row r="20">
@@ -13667,7 +13667,7 @@
         <v>316</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0985993940852531</v>
+        <v>0.101127347383383</v>
       </c>
     </row>
     <row r="21">
@@ -13675,7 +13675,7 @@
         <v>317</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0275538790963509</v>
+        <v>-0.0228596435677002</v>
       </c>
     </row>
     <row r="22">
@@ -13683,7 +13683,7 @@
         <v>318</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.167361769313469</v>
+        <v>-0.174820672774657</v>
       </c>
     </row>
     <row r="23">
@@ -13691,7 +13691,7 @@
         <v>319</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.264692288125081</v>
+        <v>-0.284204454384653</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-EIP2 | 2026-06-17 11:52:30.848148
</commit_message>
<xml_diff>
--- a/indicadores/SFE-EIP2_out.xlsx
+++ b/indicadores/SFE-EIP2_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="322">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const | td1coef</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">27/05/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1476,9 +1482,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -1489,7 +1499,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -1503,12 +1513,12 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.38543174138314</v>
+        <v>0.389319579360301</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -1519,12 +1529,12 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="E10"/>
       <c r="F10"/>
@@ -1547,7 +1557,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -1561,12 +1571,12 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.148557627265639</v>
+        <v>0.150172103878888</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -1589,7 +1599,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -1603,7 +1613,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -1617,7 +1627,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -1631,12 +1641,12 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.269781412485327</v>
+        <v>0.311768761019896</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -1647,7 +1657,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -1661,12 +1671,12 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0295660802165019</v>
+        <v>0.0297413322768401</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -1809,10 +1819,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -1825,10 +1835,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -1852,66 +1862,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>473.408721</v>
@@ -1964,7 +1974,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>509.67609</v>
@@ -2021,7 +2031,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>534.484949</v>
@@ -2078,7 +2088,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>535.318632</v>
@@ -2135,7 +2145,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>533.864619</v>
@@ -2192,7 +2202,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>522.725285</v>
@@ -2249,7 +2259,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>500.616982</v>
@@ -2306,7 +2316,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>507.807295</v>
@@ -2363,7 +2373,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>496.283071</v>
@@ -2420,7 +2430,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>504.385262</v>
@@ -2477,7 +2487,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>517.931235</v>
@@ -2534,7 +2544,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>479.85827</v>
@@ -2591,7 +2601,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>338.423937</v>
@@ -2650,7 +2660,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>368.175528</v>
@@ -2709,7 +2719,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>393.857044</v>
@@ -2768,7 +2778,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>415.258888</v>
@@ -2827,7 +2837,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>426.816954</v>
@@ -2886,7 +2896,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>417.232366</v>
@@ -2945,7 +2955,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>417.489011</v>
@@ -3004,7 +3014,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>433.39839</v>
@@ -3063,7 +3073,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>424.058105</v>
@@ -3122,7 +3132,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>415.221563</v>
@@ -3181,7 +3191,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>404.462224</v>
@@ -3240,7 +3250,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>363.801329</v>
@@ -3299,7 +3309,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>331.935393</v>
@@ -3358,7 +3368,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>363.235151</v>
@@ -3417,7 +3427,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>399.955661</v>
@@ -3476,7 +3486,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>421.306784</v>
@@ -3535,7 +3545,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>439.669383</v>
@@ -3594,7 +3604,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>431.091852</v>
@@ -3653,7 +3663,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>419.874589</v>
@@ -3712,7 +3722,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>401.556832</v>
@@ -3771,7 +3781,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>411.321515</v>
@@ -3830,7 +3840,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>428.052258</v>
@@ -3889,7 +3899,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>401.819937</v>
@@ -3948,7 +3958,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>369.520604</v>
@@ -4007,7 +4017,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>350.963803</v>
@@ -4066,7 +4076,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>370.871066</v>
@@ -4125,7 +4135,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>396.767134</v>
@@ -4184,7 +4194,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>408.772844</v>
@@ -4243,7 +4253,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>370.480018</v>
@@ -4302,7 +4312,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>427.076173</v>
@@ -4361,7 +4371,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>407.321615</v>
@@ -4420,7 +4430,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>435.049222</v>
@@ -4479,7 +4489,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>409.629796</v>
@@ -4538,7 +4548,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>420.580994</v>
@@ -4597,7 +4607,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>402.333475</v>
@@ -4656,7 +4666,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>386.969682</v>
@@ -4715,7 +4725,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>375.957336</v>
@@ -4774,7 +4784,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>392.975481</v>
@@ -4833,7 +4843,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>367.04545</v>
@@ -4892,7 +4902,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>361.310019</v>
@@ -4951,7 +4961,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>380.596106</v>
@@ -5010,7 +5020,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>383.569855</v>
@@ -5069,7 +5079,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>359.03333</v>
@@ -5128,7 +5138,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>359.636598</v>
@@ -5187,7 +5197,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>351.152484</v>
@@ -5246,7 +5256,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>358.757729</v>
@@ -5305,7 +5315,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>364.701419</v>
@@ -5364,7 +5374,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>335.706601</v>
@@ -5423,7 +5433,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>341.768896</v>
@@ -5482,7 +5492,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>351.772263</v>
@@ -5541,7 +5551,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>388.408218</v>
@@ -5600,7 +5610,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>375.762867</v>
@@ -5659,7 +5669,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>399.832795</v>
@@ -5718,7 +5728,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>376.825963</v>
@@ -5777,7 +5787,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>380.956866</v>
@@ -5836,7 +5846,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>377.548982</v>
@@ -5895,7 +5905,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>370.953081</v>
@@ -5954,7 +5964,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>388.746446</v>
@@ -6013,7 +6023,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>386.585609</v>
@@ -6072,7 +6082,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>342.777477</v>
@@ -6131,7 +6141,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>363.006602</v>
@@ -6190,7 +6200,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>393.652895</v>
@@ -6249,7 +6259,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>417.314491</v>
@@ -6308,7 +6318,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>422.199702</v>
@@ -6367,7 +6377,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>420.299275</v>
@@ -6426,7 +6436,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>393.848784</v>
@@ -6485,7 +6495,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>382.783299</v>
@@ -6544,7 +6554,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>376.486492</v>
@@ -6603,7 +6613,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>356.081395</v>
@@ -6662,7 +6672,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>384.725508</v>
@@ -6721,7 +6731,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>391.8244</v>
@@ -6780,7 +6790,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>326.468082</v>
@@ -6839,7 +6849,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>340.132077</v>
@@ -6898,7 +6908,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>360.486206</v>
@@ -6957,7 +6967,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>364.924254</v>
@@ -7016,7 +7026,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>405.979715</v>
@@ -7075,7 +7085,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>399.460014</v>
@@ -7134,7 +7144,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>384.743508</v>
@@ -7193,7 +7203,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>382.55195</v>
@@ -7252,7 +7262,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>392.900408</v>
@@ -7311,7 +7321,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>365.404312</v>
@@ -7370,7 +7380,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>382.335449</v>
@@ -7429,7 +7439,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>365.817033</v>
@@ -7488,7 +7498,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>316.255156</v>
@@ -7547,7 +7557,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>330.843236</v>
@@ -7606,7 +7616,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>342.908498</v>
@@ -7665,7 +7675,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>312.475914</v>
@@ -7724,7 +7734,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>245.673411</v>
@@ -7783,7 +7793,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>317.566413</v>
@@ -7842,7 +7852,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>319.322046</v>
@@ -7901,7 +7911,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>332.075023</v>
@@ -7960,7 +7970,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>347.503401</v>
@@ -8019,7 +8029,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>330.738112</v>
@@ -8078,7 +8088,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>348.932036</v>
@@ -8137,7 +8147,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>367.593055</v>
@@ -8196,7 +8206,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>308.480116</v>
@@ -8255,7 +8265,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>367.784947</v>
@@ -8314,7 +8324,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>367.080281</v>
@@ -8373,7 +8383,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>399.905163</v>
@@ -8432,7 +8442,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>351.423902</v>
@@ -8491,7 +8501,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>385.236403</v>
@@ -8550,7 +8560,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>379.420734</v>
@@ -8609,7 +8619,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>394.018799</v>
@@ -8668,7 +8678,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>386.055533</v>
@@ -8727,7 +8737,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>371.604464</v>
@@ -8786,7 +8796,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>383.437826</v>
@@ -8845,7 +8855,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>384.297526</v>
@@ -8904,7 +8914,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>374.436277</v>
@@ -8963,7 +8973,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>331.387524</v>
@@ -9022,7 +9032,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>332.98739</v>
@@ -9081,7 +9091,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>393.431835</v>
@@ -9140,7 +9150,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>414.625048</v>
@@ -9199,7 +9209,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>422.860595</v>
@@ -9258,7 +9268,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>412.086453</v>
@@ -9317,7 +9327,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>403.282659</v>
@@ -9376,7 +9386,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>368.792321</v>
@@ -9435,7 +9445,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>377.736312</v>
@@ -9494,7 +9504,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>394.82672</v>
@@ -9553,7 +9563,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>401.950185</v>
@@ -9612,7 +9622,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>379.460047</v>
@@ -9671,7 +9681,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>368.978742</v>
@@ -9730,7 +9740,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>299.036212</v>
@@ -9789,7 +9799,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>399.135567</v>
@@ -9848,7 +9858,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>367.821453</v>
@@ -9907,7 +9917,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>387.626802</v>
@@ -9966,7 +9976,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>374.714182</v>
@@ -10025,7 +10035,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>348.611536</v>
@@ -10084,7 +10094,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>369.798073</v>
@@ -10143,7 +10153,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>350.988516</v>
@@ -10202,7 +10212,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>352.447115</v>
@@ -10261,7 +10271,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>352.155131</v>
@@ -10320,7 +10330,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>319.339446</v>
@@ -10379,7 +10389,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>351.305725</v>
@@ -10438,7 +10448,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>311.257311</v>
@@ -10497,7 +10507,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>313.633076</v>
@@ -10556,7 +10566,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>331.816929</v>
@@ -10615,7 +10625,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>352.894679</v>
@@ -10674,7 +10684,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>313.058211</v>
@@ -10733,7 +10743,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>328.724527</v>
@@ -10792,7 +10802,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>332.108764</v>
@@ -10851,7 +10861,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>351.212435</v>
@@ -10910,7 +10920,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>374.624636</v>
@@ -10969,7 +10979,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>343.648964</v>
@@ -11028,7 +11038,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>291.600981</v>
@@ -11087,7 +11097,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>350.630642</v>
@@ -11146,7 +11156,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>333.429285</v>
@@ -11205,7 +11215,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>341.22981</v>
@@ -11264,7 +11274,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>303.130568</v>
@@ -11323,7 +11333,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>347.61999</v>
@@ -11382,7 +11392,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>324.466315</v>
@@ -11441,7 +11451,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>336.428761</v>
@@ -11500,7 +11510,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>337.259481</v>
@@ -11559,7 +11569,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>317.878281</v>
@@ -11618,7 +11628,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>327.975055</v>
@@ -11677,7 +11687,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>327.255348</v>
@@ -11736,7 +11746,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>297.965411</v>
@@ -11795,7 +11805,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>311.307882</v>
@@ -11854,7 +11864,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>296.8625</v>
@@ -11913,7 +11923,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>355.270003</v>
@@ -11972,7 +11982,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>342.57694</v>
@@ -12031,7 +12041,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2"/>
       <c r="C174" s="3" t="n">
@@ -12064,7 +12074,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2"/>
       <c r="C175" s="3" t="n">
@@ -12097,7 +12107,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2"/>
       <c r="C176" s="3" t="n">
@@ -12130,7 +12140,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2"/>
       <c r="C177" s="3" t="n">
@@ -12163,7 +12173,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2"/>
       <c r="C178" s="3" t="n">
@@ -12196,7 +12206,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2"/>
       <c r="C179" s="3" t="n">
@@ -12229,7 +12239,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2"/>
       <c r="C180" s="3" t="n">
@@ -12262,7 +12272,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2"/>
       <c r="C181" s="3" t="n">
@@ -12295,7 +12305,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2"/>
       <c r="C182" s="3" t="n">
@@ -12328,7 +12338,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2"/>
       <c r="C183" s="3" t="n">
@@ -12361,7 +12371,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2"/>
       <c r="C184" s="3" t="n">
@@ -12394,7 +12404,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2"/>
       <c r="C185" s="3" t="n">
@@ -12427,7 +12437,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2"/>
       <c r="C186" s="3"/>
@@ -12450,7 +12460,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2"/>
       <c r="C187" s="3"/>
@@ -12473,7 +12483,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2"/>
       <c r="C188" s="3"/>
@@ -12496,7 +12506,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2"/>
       <c r="C189" s="3"/>
@@ -12519,7 +12529,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2"/>
       <c r="C190" s="3"/>
@@ -12542,7 +12552,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2"/>
       <c r="C191" s="3"/>
@@ -12565,7 +12575,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2"/>
       <c r="C192" s="3"/>
@@ -12588,7 +12598,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2"/>
       <c r="C193" s="3"/>
@@ -12611,7 +12621,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2"/>
       <c r="C194" s="3"/>
@@ -12634,7 +12644,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2"/>
       <c r="C195" s="3"/>
@@ -12657,7 +12667,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2"/>
       <c r="C196" s="3"/>
@@ -12680,7 +12690,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2"/>
       <c r="C197" s="3"/>
@@ -12703,7 +12713,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2"/>
       <c r="C198" s="3"/>
@@ -12726,7 +12736,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2"/>
       <c r="C199" s="3"/>
@@ -12749,7 +12759,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2"/>
       <c r="C200" s="3"/>
@@ -12772,7 +12782,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2"/>
       <c r="C201" s="3"/>
@@ -12795,7 +12805,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2"/>
       <c r="C202" s="3"/>
@@ -12818,7 +12828,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2"/>
       <c r="C203" s="3"/>
@@ -12841,7 +12851,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2"/>
       <c r="C204" s="3"/>
@@ -12864,7 +12874,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2"/>
       <c r="C205" s="3"/>
@@ -12887,7 +12897,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2"/>
       <c r="C206" s="3"/>
@@ -12910,7 +12920,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2"/>
       <c r="C207" s="3"/>
@@ -12933,7 +12943,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2"/>
       <c r="C208" s="3"/>
@@ -12956,7 +12966,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2"/>
       <c r="C209" s="3"/>
@@ -12979,7 +12989,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2"/>
       <c r="C210" s="3"/>
@@ -13002,7 +13012,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2"/>
       <c r="C211" s="3"/>
@@ -13025,7 +13035,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2"/>
       <c r="C212" s="3"/>
@@ -13048,7 +13058,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2"/>
       <c r="C213" s="3"/>
@@ -13071,7 +13081,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2"/>
       <c r="C214" s="3"/>
@@ -13094,7 +13104,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2"/>
       <c r="C215" s="3"/>
@@ -13117,7 +13127,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2"/>
       <c r="C216" s="3"/>
@@ -13140,7 +13150,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2"/>
       <c r="C217" s="3"/>
@@ -13163,7 +13173,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2"/>
       <c r="C218" s="3"/>
@@ -13186,7 +13196,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2"/>
       <c r="C219" s="3"/>
@@ -13209,7 +13219,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2"/>
       <c r="C220" s="3"/>
@@ -13232,7 +13242,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2"/>
       <c r="C221" s="3"/>
@@ -13255,7 +13265,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2"/>
       <c r="C222" s="3"/>
@@ -13278,7 +13288,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2"/>
       <c r="C223" s="3"/>
@@ -13301,7 +13311,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2"/>
       <c r="C224" s="3"/>
@@ -13324,7 +13334,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2"/>
       <c r="C225" s="3"/>
@@ -13347,7 +13357,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2"/>
       <c r="C226" s="3"/>
@@ -13370,7 +13380,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2"/>
       <c r="C227" s="3"/>
@@ -13393,7 +13403,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2"/>
       <c r="C228" s="3"/>
@@ -13416,7 +13426,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2"/>
       <c r="C229" s="3"/>
@@ -13450,97 +13460,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -13564,7 +13574,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -13574,160 +13584,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.183904276747433</v>
+        <v>-0.181721112584506</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.19190593823227</v>
+        <v>-0.194461237804537</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.197011866063527</v>
+        <v>-0.204126315284641</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>-0.185909565337546</v>
+        <v>-0.187246833554567</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.119778182920673</v>
+        <v>-0.116484588219302</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.00738861721474648</v>
+        <v>0.0050628623358604</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.137430860880173</v>
+        <v>0.13528762392719</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.271281895268374</v>
+        <v>0.276564847661299</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.384730578131587</v>
+        <v>0.389319579360301</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.38543174138314</v>
+        <v>0.387520456077983</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.328189187827614</v>
+        <v>0.333491909451648</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.302556033305567</v>
+        <v>0.310379349874548</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.277056073663907</v>
+        <v>0.284824307731637</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.231917841732091</v>
+        <v>0.234458917927675</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.181378412877099</v>
+        <v>0.179613211971548</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.104114582708344</v>
+        <v>0.10234684727086</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>-0.0171693103863784</v>
+        <v>-0.0187333850004688</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>-0.170330044827159</v>
+        <v>-0.169244177695529</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>-0.284156035269357</v>
+        <v>-0.280199768676928</v>
       </c>
     </row>
     <row r="24">

</xml_diff>